<commit_message>
Recalculate fantasy points with correct league scoring
Dot balls +2, economy bonuses doubled, wicket hauls doubled, duck -4.
Bowlers jump 15-20 pts avg. Updated team comparison Excel.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Draft_Teams_Comparison.xlsx
+++ b/output/Draft_Teams_Comparison.xlsx
@@ -673,13 +673,13 @@
         <v>7567</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>8553</v>
+        <v>8565</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>13</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>657.9</v>
+        <v>658.8</v>
       </c>
     </row>
     <row r="8">
@@ -5721,10 +5721,10 @@
       <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="14" t="inlineStr"/>
       <c r="F14" s="12" t="n">
-        <v>57.6</v>
+        <v>60</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="H14" s="12" t="n">
         <v>5</v>
@@ -5830,7 +5830,7 @@
         </is>
       </c>
       <c r="G18" s="19" t="n">
-        <v>8553</v>
+        <v>8565</v>
       </c>
       <c r="K18" s="19" t="n">
         <v>7567</v>
@@ -5843,7 +5843,7 @@
         </is>
       </c>
       <c r="F19" s="19" t="n">
-        <v>657.9</v>
+        <v>658.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>